<commit_message>
my maps tugmasi qoshildi
</commit_message>
<xml_diff>
--- a/dorixonalar.xlsx
+++ b/dorixonalar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\gpp\dorixona-bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8354F957-ACE4-4566-B1F8-403E28ACD442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADDC089-6E55-4239-8310-ED8B666D8B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="493">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1186" uniqueCount="499">
   <si>
     <t>Filial №</t>
   </si>
@@ -1499,6 +1499,24 @@
   </si>
   <si>
     <t>1-сон шахар клиник шифохонаси, тугрукхона рупараси</t>
+  </si>
+  <si>
+    <t>41.204489</t>
+  </si>
+  <si>
+    <t>69.227648</t>
+  </si>
+  <si>
+    <t>69.345592</t>
+  </si>
+  <si>
+    <t>41.285519</t>
+  </si>
+  <si>
+    <t>41.295130</t>
+  </si>
+  <si>
+    <t>69.334867</t>
   </si>
 </sst>
 </file>
@@ -2635,11 +2653,11 @@
       <c r="N18" t="s">
         <v>90</v>
       </c>
-      <c r="O18">
-        <v>41.303612000000001</v>
-      </c>
-      <c r="P18">
-        <v>69.303685999999999</v>
+      <c r="O18" t="s">
+        <v>497</v>
+      </c>
+      <c r="P18" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
@@ -4785,11 +4803,11 @@
       <c r="N67" t="s">
         <v>291</v>
       </c>
-      <c r="O67">
-        <v>41.285631000000002</v>
-      </c>
-      <c r="P67">
-        <v>69.346453999999994</v>
+      <c r="O67" t="s">
+        <v>496</v>
+      </c>
+      <c r="P67" t="s">
+        <v>495</v>
       </c>
     </row>
     <row r="68" spans="1:16" x14ac:dyDescent="0.25">
@@ -6061,11 +6079,11 @@
       <c r="N96" t="s">
         <v>409</v>
       </c>
-      <c r="O96">
-        <v>41.20431</v>
-      </c>
-      <c r="P96">
-        <v>69.228810999999993</v>
+      <c r="O96" t="s">
+        <v>493</v>
+      </c>
+      <c r="P96" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="97" spans="1:16" x14ac:dyDescent="0.25">

</xml_diff>